<commit_message>
faculty availability feature added and working
</commit_message>
<xml_diff>
--- a/TIME TABLE SAMPLE DATA/faculty-availability-template.xlsx
+++ b/TIME TABLE SAMPLE DATA/faculty-availability-template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ganig\Desktop\Time_Table_\TIME TABLE SAMPLE DATA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5afc8f5c19c83632/Desktop/Timetable/TIME TABLE SAMPLE DATA/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAF29F99-14D0-464F-A2DF-6ABDA197F981}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -422,9 +422,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -447,7 +447,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>14</v>
       </c>

</xml_diff>